<commit_message>
Mejorar importacion de productos con wizard, mapeo de columnas y validacion previa.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/plantilla_alcentimo.xlsx
+++ b/public/plantilla_alcentimo.xlsx
@@ -403,8 +403,8 @@
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="42.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="42.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,10 +421,10 @@
         <v>stock</v>
       </c>
       <c r="E1" t="str">
+        <v>categoria</v>
+      </c>
+      <c r="F1" t="str">
         <v>url_imagen</v>
-      </c>
-      <c r="F1" t="str">
-        <v>categoria</v>
       </c>
     </row>
     <row r="2">
@@ -441,10 +441,10 @@
         <v>15</v>
       </c>
       <c r="E2" t="str">
+        <v>camisas</v>
+      </c>
+      <c r="F2" t="str">
         <v>https://ejemplo.com/imagenes/camisa-oxford.jpg</v>
-      </c>
-      <c r="F2" t="str">
-        <v>camisas</v>
       </c>
     </row>
     <row r="3">
@@ -461,10 +461,10 @@
         <v>8</v>
       </c>
       <c r="E3" t="str">
+        <v>pantalones</v>
+      </c>
+      <c r="F3" t="str">
         <v/>
-      </c>
-      <c r="F3" t="str">
-        <v>pantalones</v>
       </c>
     </row>
   </sheetData>

</xml_diff>